<commit_message>
feat(F-NAR-016): TREE-DIF-039 passe agent après apply
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-DIF-039.xlsx
+++ b/stories/arbres/TREE-DIF-039.xlsx
@@ -6923,12 +6923,12 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Sur le dos. Oui. Le sac à pois tient une ombre ronde. Je vois les pois ! Ne le lance pas encore. Aniss a les cheveux tout courts. Une mèche saute quand il respire. Ça sent déjà le trottoir chaud. Vos mains, sur le sac ? Oui, papa.</t>
+          <t>Sur le dos. Oui. Le sac à pois tient une ombre ronde. Je vois les pois ! On le garde pour le portail. Aniss a les cheveux tout courts. Une mèche saute quand il respire. Ça sent déjà le trottoir chaud. Vos mains, sur le sac ? Oui, papa.</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Sur le dos. Oui. Le sac à pois tient une ombre ronde. Je vois les pois ! Ne le lance pas encore. Aniss a les cheveux tout courts. Une mèche saute quand il respire. Ça sent déjà le trottoir chaud. Vos mains, sur le sac ? Oui, papa.</t>
+          <t>Sur le dos. Oui. Le sac à pois tient une ombre ronde. Je vois les pois ! On le garde pour le portail. Aniss a les cheveux tout courts. Une mèche saute quand il respire. Ça sent déjà le trottoir chaud. Vos mains, sur le sac ? Oui, papa.</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -7071,7 +7071,7 @@
 papa|Oui.
 narrateur|Le sac à pois tient une ombre ronde.
 copain|Je vois les pois !
-enfant-m|Ne le lance pas encore.
+enfant-m|On le garde pour le portail.
 narrateur|Aniss a les cheveux tout courts.
 narrateur|Une mèche saute quand il respire.
 maman|Ça sent déjà le trottoir chaud.
@@ -10134,12 +10134,12 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Le sac à pois fait un rond sur le muret. Ici, ça mène au portail, Aniss. Je vais plus loin, encore ! Le muret renvoie chaque pas, tout fort. Aniss court après le sac, plus loin. Le sac à pois attend au bord, un peu seule. Son élan remplit tout le mur. Toi tu vas plus loin, lui plus vite. On rebondit comment, alors ? Vous trouvez, tous les deux ?</t>
+          <t>Le sac à pois s'appuie contre le muret. Ici, ça mène au portail, Aniss. Je vais plus loin, encore ! Le muret renvoie chaque pas, tout fort. Aniss court après le sac, plus loin. Le sac à pois attend au bord, un peu seule. Son élan remplit tout le mur. Toi tu vas plus loin, lui plus vite. On rebondit comment, alors ? Vous trouvez, tous les deux ?</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Le sac à pois fait un rond sur le muret. Ici, ça mène au portail, Aniss. Je vais plus loin, encore ! Le muret renvoie chaque pas, tout fort. Aniss court après le sac, plus loin. Le sac à pois attend au bord, un peu seule. Son élan remplit tout le mur. Toi tu vas plus loin, lui plus vite. On rebondit comment, alors ? Vous trouvez, tous les deux ?</t>
+          <t>Le sac à pois s'appuie contre le muret. Ici, ça mène au portail, Aniss. Je vais plus loin, encore ! Le muret renvoie chaque pas, tout fort. Aniss court après le sac, plus loin. Le sac à pois attend au bord, un peu seule. Son élan remplit tout le mur. Toi tu vas plus loin, lui plus vite. On rebondit comment, alors ? Vous trouvez, tous les deux ?</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -10274,7 +10274,7 @@
       <c r="AV52" s="2" t="inlineStr"/>
       <c r="AW52" t="inlineStr">
         <is>
-          <t>narrateur|Le sac à pois fait un rond sur le muret.
+          <t>narrateur|Le sac à pois s'appuie contre le muret.
 enfant-m|Ici, ça mène au portail, Aniss.
 copain|Je vais plus loin, encore !
 narrateur|Le muret renvoie chaque pas, tout fort.
@@ -15125,12 +15125,12 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>La gourde bleue pose un pied près du muret. Ici, ça mène au portail, Aniss. Je vais plus loin, encore ! Le muret renvoie chaque pas, tout fort. Aniss chasse la gourde, le muret le suit. La gourde bleue attend au bord, un peu seule. Son élan remplit tout le mur. Toi tu vas plus loin, lui plus vite. On rebondit comment, alors ? Vous trouvez, tous les deux ?</t>
+          <t>La gourde bleue s'arrête près du muret. Ici, ça mène au portail, Aniss. Je vais plus loin, encore ! Le muret renvoie chaque pas, tout fort. Aniss court, la gourde reste contre la pierre. La gourde bleue attend au bord, un peu seule. Son élan remplit tout le mur. Toi tu vas plus loin, lui plus vite. On rebondit comment, alors ? Vous trouvez, tous les deux ?</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>La gourde bleue pose un pied près du muret. Ici, ça mène au portail, Aniss. Je vais plus loin, encore ! Le muret renvoie chaque pas, tout fort. Aniss chasse la gourde, le muret le suit. La gourde bleue attend au bord, un peu seule. Son élan remplit tout le mur. Toi tu vas plus loin, lui plus vite. On rebondit comment, alors ? Vous trouvez, tous les deux ?</t>
+          <t>La gourde bleue s'arrête près du muret. Ici, ça mène au portail, Aniss. Je vais plus loin, encore ! Le muret renvoie chaque pas, tout fort. Aniss court, la gourde reste contre la pierre. La gourde bleue attend au bord, un peu seule. Son élan remplit tout le mur. Toi tu vas plus loin, lui plus vite. On rebondit comment, alors ? Vous trouvez, tous les deux ?</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -15265,11 +15265,11 @@
       <c r="AV80" s="2" t="inlineStr"/>
       <c r="AW80" t="inlineStr">
         <is>
-          <t>narrateur|La gourde bleue pose un pied près du muret.
+          <t>narrateur|La gourde bleue s'arrête près du muret.
 enfant-m|Ici, ça mène au portail, Aniss.
 copain|Je vais plus loin, encore !
 narrateur|Le muret renvoie chaque pas, tout fort.
-narrateur|Aniss chasse la gourde, le muret le suit.
+narrateur|Aniss court, la gourde reste contre la pierre.
 narrateur|La gourde bleue attend au bord, un peu seule.
 maman|Son élan remplit tout le mur.
 papa|Toi tu vas plus loin, lui plus vite.
@@ -16537,7 +16537,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -16580,6 +16580,13 @@
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>